<commit_message>
feat: verify rule CG0089 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000016/negative/01/data/unit-test-coreid-CG0089-negative.xlsx
+++ b/rules/CORE-000016/negative/01/data/unit-test-coreid-CG0089-negative.xlsx
@@ -48,7 +48,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,6 +130,10 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -699,7 +709,8 @@
           <t>CIGARETTES</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -729,7 +740,8 @@
           <t>CAFFEINE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -759,7 +771,8 @@
           <t>TOBACCO</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1145,8 +1158,8 @@
           <t>Collecting</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1176,8 +1189,8 @@
           <t>Extracting</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1207,8 +1220,8 @@
           <t>Shipping</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1238,8 +1251,8 @@
           <t>Aliquoting</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1417,7 +1430,8 @@
           <t>Rash</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1447,7 +1461,8 @@
           <t>Wheezing</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1477,7 +1492,8 @@
           <t>Edema</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1507,7 +1523,8 @@
           <t>Conjunctivitis</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2255,7 +2272,8 @@
           <t>HOSPITAL</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2285,7 +2303,8 @@
           <t>NURSING HOME</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2315,7 +2334,8 @@
           <t>GENERAL WARD</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2345,7 +2365,8 @@
           <t>INTENSIVE CARE</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2523,7 +2544,8 @@
           <t>ASTHMA</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2553,7 +2575,8 @@
           <t>CONGESTIVE HEART FAILURE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2583,7 +2606,8 @@
           <t>BROKEN LEG</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2613,7 +2637,8 @@
           <t>HEADACHES</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2824,7 +2849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2856,6 +2881,1740 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>11</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>12</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>13</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>14</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>15</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>16</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>16</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>17</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>17</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>6</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>18</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>18</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>19</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>20</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>6</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>20</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>21</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>7</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>21</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>22</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>8</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>22</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>23</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>23</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>24</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>6</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>24</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>25</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>7</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>25</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>7</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>26</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>8</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>26</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>8</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>27</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>5</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>27</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>5</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>28</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>6</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>28</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>6</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>29</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>7</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>29</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>7</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>30</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>8</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>8</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>31</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>5</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>31</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>5</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>32</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>32</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>6</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>33</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>7</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>33</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>7</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>34</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>8</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>34</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -3031,7 +4790,8 @@
           <t>Buprenorphine</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3061,7 +4821,8 @@
           <t>Minims Proxymetacaine</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3091,7 +4852,8 @@
           <t>Meloxicam</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3269,7 +5031,8 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3299,7 +5062,8 @@
           <t>METAMUCIL</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3329,7 +5093,8 @@
           <t>HYDROCORTISONE, TOPICAL</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3507,7 +5272,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3537,7 +5303,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3567,7 +5334,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4025,7 +5793,8 @@
           <t>SNACK</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4055,7 +5824,8 @@
           <t>NUTRITIONAL DRINK</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -4085,7 +5855,8 @@
           <t>WILD MUSHROOMS</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4263,7 +6034,8 @@
           <t>Wisdom Teeth Extraction</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4293,7 +6065,8 @@
           <t>Endoscopy</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -4323,7 +6096,8 @@
           <t>Heart Transplant</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>